<commit_message>
Remove screening sheet, add MedGemma-Critic link
</commit_message>
<xml_diff>
--- a/SLM_Review_Dataset.xlsx
+++ b/SLM_Review_Dataset.xlsx
@@ -10,8 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Included_102" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded_18" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRISMA_Flow" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Included_102'!$A$1:$Z$103</definedName>
@@ -26,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,10 +64,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <i val="1"/>
@@ -145,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -181,11 +176,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -193,6 +183,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -10307,7 +10298,11 @@
           <t>2025 International Conference on Digital Image Computing: Techniques and Applications (DICTA)</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>https://ieeexplore.ieee.org/abstract/document/11302446</t>
+        </is>
+      </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
           <t>Peer-reviewed</t>
@@ -12668,25 +12663,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId101"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13977,243 +13973,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Inter-rater agreement (two independent reviewers)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>Enter the 2×2 decision counts in the white cells; agreement and Cohen's kappa are computed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>Title and abstract screening</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr"/>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Reviewer B: Include</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Reviewer B: Exclude</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Reviewer A: Include</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="18">
-        <f>B6+C6</f>
-        <v/>
-      </c>
-      <c r="F6" s="17" t="inlineStr">
-        <is>
-          <t>Observed agreement (pₒ)</t>
-        </is>
-      </c>
-      <c r="G6" s="19">
-        <f>(B6+C7)/D8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Reviewer A: Exclude</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="18">
-        <f>B7+C7</f>
-        <v/>
-      </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>Expected agreement (pₑ)</t>
-        </is>
-      </c>
-      <c r="G7" s="19">
-        <f>(D6*B8+D7*C8)/D8^2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B8" s="18">
-        <f>B6+B7</f>
-        <v/>
-      </c>
-      <c r="C8" s="18">
-        <f>C6+C7</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>D6+D7</f>
-        <v/>
-      </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>Cohen's κ</t>
-        </is>
-      </c>
-      <c r="G8" s="20">
-        <f>(G6-G7)/(1-G7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>Full-text assessment</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr"/>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>Reviewer B: Include</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>Reviewer B: Exclude</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>Reviewer A: Include</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="18">
-        <f>B14+C14</f>
-        <v/>
-      </c>
-      <c r="F14" s="17" t="inlineStr">
-        <is>
-          <t>Observed agreement (pₒ)</t>
-        </is>
-      </c>
-      <c r="G14" s="19">
-        <f>(B14+C15)/D16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>Reviewer A: Exclude</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="18">
-        <f>B15+C15</f>
-        <v/>
-      </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>Expected agreement (pₑ)</t>
-        </is>
-      </c>
-      <c r="G15" s="19">
-        <f>(D14*B16+D15*C16)/D16^2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B16" s="18">
-        <f>B14+B15</f>
-        <v/>
-      </c>
-      <c r="C16" s="18">
-        <f>C14+C15</f>
-        <v/>
-      </c>
-      <c r="D16" s="18">
-        <f>D14+D15</f>
-        <v/>
-      </c>
-      <c r="F16" s="17" t="inlineStr">
-        <is>
-          <t>Cohen's κ</t>
-        </is>
-      </c>
-      <c r="G16" s="20">
-        <f>(G14-G15)/(1-G15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>Disagreements at both stages were resolved by the senior reviewer after discussion. Data extraction was performed by one reviewer and checked in full by the senior reviewer.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -14275,7 +14034,7 @@
         <f>COUNTIF(Included_102!$E$2:$E$103,2022)</f>
         <v/>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="17">
         <f>B6/B$11</f>
         <v/>
       </c>
@@ -14290,7 +14049,7 @@
         <f>COUNTIF(Included_102!$E$2:$E$103,2023)</f>
         <v/>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="17">
         <f>B7/B$11</f>
         <v/>
       </c>
@@ -14305,7 +14064,7 @@
         <f>COUNTIF(Included_102!$E$2:$E$103,2024)</f>
         <v/>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="17">
         <f>B8/B$11</f>
         <v/>
       </c>
@@ -14320,7 +14079,7 @@
         <f>COUNTIF(Included_102!$E$2:$E$103,2025)</f>
         <v/>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="17">
         <f>B9/B$11</f>
         <v/>
       </c>
@@ -14335,22 +14094,22 @@
         <f>COUNTIF(Included_102!$E$2:$E$103,2026)</f>
         <v/>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="17">
         <f>B10/B$11</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B11" s="23">
+      <c r="B11" s="18">
         <f>SUM(B6:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="19">
         <f>B11/B11</f>
         <v/>
       </c>
@@ -14380,7 +14139,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Lightweight</t>
         </is>
@@ -14389,13 +14148,13 @@
         <f>COUNTIF(Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="17">
         <f>B16/B$22</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="26" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Compact</t>
         </is>
@@ -14404,13 +14163,13 @@
         <f>COUNTIF(Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="17">
         <f>B17/B$22</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -14419,13 +14178,13 @@
         <f>COUNTIF(Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="17">
         <f>B18/B$22</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Higher</t>
         </is>
@@ -14434,7 +14193,7 @@
         <f>COUNTIF(Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="17">
         <f>B19/B$22</f>
         <v/>
       </c>
@@ -14449,7 +14208,7 @@
         <f>COUNTIF(Included_102!$R$2:$R$103,"Mixed")</f>
         <v/>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="17">
         <f>B20/B$22</f>
         <v/>
       </c>
@@ -14464,22 +14223,22 @@
         <f>COUNTIF(Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="17">
         <f>B21/B$22</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B22" s="23">
+      <c r="B22" s="18">
         <f>SUM(B16:B21)</f>
         <v/>
       </c>
-      <c r="C22" s="24">
+      <c r="C22" s="19">
         <f>B22/B22</f>
         <v/>
       </c>
@@ -14518,7 +14277,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Natural Language Processing")</f>
         <v/>
       </c>
-      <c r="C27" s="22">
+      <c r="C27" s="17">
         <f>B27/B$37</f>
         <v/>
       </c>
@@ -14533,7 +14292,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Agentic AI Applications")</f>
         <v/>
       </c>
-      <c r="C28" s="22">
+      <c r="C28" s="17">
         <f>B28/B$37</f>
         <v/>
       </c>
@@ -14548,7 +14307,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Coding &amp; Software Eng.")</f>
         <v/>
       </c>
-      <c r="C29" s="22">
+      <c r="C29" s="17">
         <f>B29/B$37</f>
         <v/>
       </c>
@@ -14563,7 +14322,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Healthcare &amp; Biomedical")</f>
         <v/>
       </c>
-      <c r="C30" s="22">
+      <c r="C30" s="17">
         <f>B30/B$37</f>
         <v/>
       </c>
@@ -14578,7 +14337,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Robotics &amp; Real-Time")</f>
         <v/>
       </c>
-      <c r="C31" s="22">
+      <c r="C31" s="17">
         <f>B31/B$37</f>
         <v/>
       </c>
@@ -14593,7 +14352,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Audio &amp; Speech")</f>
         <v/>
       </c>
-      <c r="C32" s="22">
+      <c r="C32" s="17">
         <f>B32/B$37</f>
         <v/>
       </c>
@@ -14608,7 +14367,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Emerging &amp; Cross-Cutting")</f>
         <v/>
       </c>
-      <c r="C33" s="22">
+      <c r="C33" s="17">
         <f>B33/B$37</f>
         <v/>
       </c>
@@ -14623,7 +14382,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Sustainability, Materials &amp; Life Sci.")</f>
         <v/>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="17">
         <f>B34/B$37</f>
         <v/>
       </c>
@@ -14638,7 +14397,7 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"Law &amp; Finance")</f>
         <v/>
       </c>
-      <c r="C35" s="22">
+      <c r="C35" s="17">
         <f>B35/B$37</f>
         <v/>
       </c>
@@ -14653,33 +14412,33 @@
         <f>COUNTIF(Included_102!$U$2:$U$103,"General (techniques / evaluation)")</f>
         <v/>
       </c>
-      <c r="C36" s="22">
+      <c r="C36" s="17">
         <f>B36/B$37</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B37" s="23">
+      <c r="B37" s="18">
         <f>SUM(B27:B36)</f>
         <v/>
       </c>
-      <c r="C37" s="24">
+      <c r="C37" s="19">
         <f>B37/B37</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>Domain-specific (Table 4)</t>
         </is>
       </c>
-      <c r="B38" s="29">
+      <c r="B38" s="25">
         <f>COUNTIF(Included_102!$U$2:$U$103,"&lt;&gt;General (techniques / evaluation)")</f>
         <v/>
       </c>
@@ -14718,7 +14477,7 @@
         <f>COUNTIF(Included_102!$H$2:$H$103,"Peer-reviewed")</f>
         <v/>
       </c>
-      <c r="C44" s="22">
+      <c r="C44" s="17">
         <f>B44/B$46</f>
         <v/>
       </c>
@@ -14733,22 +14492,22 @@
         <f>COUNTIF(Included_102!$H$2:$H$103,"Preprint")</f>
         <v/>
       </c>
-      <c r="C45" s="22">
+      <c r="C45" s="17">
         <f>B45/B$46</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="23" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B46" s="23">
+      <c r="B46" s="18">
         <f>SUM(B44:B45)</f>
         <v/>
       </c>
-      <c r="C46" s="24">
+      <c r="C46" s="19">
         <f>B46/B46</f>
         <v/>
       </c>
@@ -14778,7 +14537,7 @@
           <t>(a) Code or weights released</t>
         </is>
       </c>
-      <c r="B51" s="29">
+      <c r="B51" s="25">
         <f>COUNTIF(Included_102!$K$2:$K$103,"Yes")</f>
         <v/>
       </c>
@@ -14789,7 +14548,7 @@
           <t>(b) ≥ 5 citations</t>
         </is>
       </c>
-      <c r="B52" s="29">
+      <c r="B52" s="25">
         <f>COUNTIF(Included_102!$L$2:$L$103,"Yes")</f>
         <v/>
       </c>
@@ -14800,7 +14559,7 @@
           <t>(c) Technical report of a released model</t>
         </is>
       </c>
-      <c r="B53" s="29">
+      <c r="B53" s="25">
         <f>COUNTIF(Included_102!$M$2:$M$103,"Yes")</f>
         <v/>
       </c>
@@ -14830,7 +14589,7 @@
           <t>Studies that use at least one 7–10B model</t>
         </is>
       </c>
-      <c r="B58" s="29">
+      <c r="B58" s="25">
         <f>COUNTIF(Included_102!$T$2:$T$103,"Yes")</f>
         <v/>
       </c>
@@ -14841,7 +14600,7 @@
           <t>Studies that use only 7–10B models</t>
         </is>
       </c>
-      <c r="B59" s="29">
+      <c r="B59" s="25">
         <f>COUNTIF(Included_102!$S$2:$S$103,"Higher")</f>
         <v/>
       </c>
@@ -14901,19 +14660,19 @@
           <t>Natural Language Processing</t>
         </is>
       </c>
-      <c r="B64" s="25">
+      <c r="B64" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Natural Language Processing",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C64" s="26">
+      <c r="C64" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Natural Language Processing",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D64" s="27">
+      <c r="D64" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Natural Language Processing",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E64" s="28">
+      <c r="E64" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Natural Language Processing",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -14925,7 +14684,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Natural Language Processing",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H64" s="30">
+      <c r="H64" s="26">
         <f>SUM(B64:G64)</f>
         <v/>
       </c>
@@ -14936,19 +14695,19 @@
           <t>Agentic AI Applications</t>
         </is>
       </c>
-      <c r="B65" s="25">
+      <c r="B65" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Agentic AI Applications",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C65" s="26">
+      <c r="C65" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Agentic AI Applications",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D65" s="27">
+      <c r="D65" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Agentic AI Applications",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E65" s="28">
+      <c r="E65" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Agentic AI Applications",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -14960,7 +14719,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Agentic AI Applications",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H65" s="30">
+      <c r="H65" s="26">
         <f>SUM(B65:G65)</f>
         <v/>
       </c>
@@ -14971,19 +14730,19 @@
           <t>Coding &amp; Software Eng.</t>
         </is>
       </c>
-      <c r="B66" s="25">
+      <c r="B66" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Coding &amp; Software Eng.",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C66" s="26">
+      <c r="C66" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Coding &amp; Software Eng.",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D66" s="27">
+      <c r="D66" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Coding &amp; Software Eng.",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E66" s="28">
+      <c r="E66" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Coding &amp; Software Eng.",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -14995,7 +14754,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Coding &amp; Software Eng.",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H66" s="30">
+      <c r="H66" s="26">
         <f>SUM(B66:G66)</f>
         <v/>
       </c>
@@ -15006,19 +14765,19 @@
           <t>Healthcare &amp; Biomedical</t>
         </is>
       </c>
-      <c r="B67" s="25">
+      <c r="B67" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Healthcare &amp; Biomedical",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C67" s="26">
+      <c r="C67" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Healthcare &amp; Biomedical",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D67" s="27">
+      <c r="D67" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Healthcare &amp; Biomedical",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E67" s="28">
+      <c r="E67" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Healthcare &amp; Biomedical",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -15030,7 +14789,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Healthcare &amp; Biomedical",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H67" s="30">
+      <c r="H67" s="26">
         <f>SUM(B67:G67)</f>
         <v/>
       </c>
@@ -15041,19 +14800,19 @@
           <t>Robotics &amp; Real-Time</t>
         </is>
       </c>
-      <c r="B68" s="25">
+      <c r="B68" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Robotics &amp; Real-Time",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C68" s="26">
+      <c r="C68" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Robotics &amp; Real-Time",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D68" s="27">
+      <c r="D68" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Robotics &amp; Real-Time",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E68" s="28">
+      <c r="E68" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Robotics &amp; Real-Time",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -15065,7 +14824,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Robotics &amp; Real-Time",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H68" s="30">
+      <c r="H68" s="26">
         <f>SUM(B68:G68)</f>
         <v/>
       </c>
@@ -15076,19 +14835,19 @@
           <t>Audio &amp; Speech</t>
         </is>
       </c>
-      <c r="B69" s="25">
+      <c r="B69" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Audio &amp; Speech",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C69" s="26">
+      <c r="C69" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Audio &amp; Speech",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D69" s="27">
+      <c r="D69" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Audio &amp; Speech",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E69" s="28">
+      <c r="E69" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Audio &amp; Speech",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -15100,7 +14859,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Audio &amp; Speech",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H69" s="30">
+      <c r="H69" s="26">
         <f>SUM(B69:G69)</f>
         <v/>
       </c>
@@ -15111,19 +14870,19 @@
           <t>Emerging &amp; Cross-Cutting</t>
         </is>
       </c>
-      <c r="B70" s="25">
+      <c r="B70" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Emerging &amp; Cross-Cutting",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C70" s="26">
+      <c r="C70" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Emerging &amp; Cross-Cutting",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D70" s="27">
+      <c r="D70" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Emerging &amp; Cross-Cutting",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E70" s="28">
+      <c r="E70" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Emerging &amp; Cross-Cutting",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -15135,7 +14894,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Emerging &amp; Cross-Cutting",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H70" s="30">
+      <c r="H70" s="26">
         <f>SUM(B70:G70)</f>
         <v/>
       </c>
@@ -15146,19 +14905,19 @@
           <t>Sustainability, Materials &amp; Life Sci.</t>
         </is>
       </c>
-      <c r="B71" s="25">
+      <c r="B71" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Sustainability, Materials &amp; Life Sci.",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C71" s="26">
+      <c r="C71" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Sustainability, Materials &amp; Life Sci.",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D71" s="27">
+      <c r="D71" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Sustainability, Materials &amp; Life Sci.",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E71" s="28">
+      <c r="E71" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Sustainability, Materials &amp; Life Sci.",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -15170,7 +14929,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Sustainability, Materials &amp; Life Sci.",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H71" s="30">
+      <c r="H71" s="26">
         <f>SUM(B71:G71)</f>
         <v/>
       </c>
@@ -15181,19 +14940,19 @@
           <t>Law &amp; Finance</t>
         </is>
       </c>
-      <c r="B72" s="25">
+      <c r="B72" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Law &amp; Finance",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C72" s="26">
+      <c r="C72" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Law &amp; Finance",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D72" s="27">
+      <c r="D72" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Law &amp; Finance",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E72" s="28">
+      <c r="E72" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Law &amp; Finance",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -15205,7 +14964,7 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"Law &amp; Finance",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H72" s="30">
+      <c r="H72" s="26">
         <f>SUM(B72:G72)</f>
         <v/>
       </c>
@@ -15216,19 +14975,19 @@
           <t>General (techniques / evaluation)</t>
         </is>
       </c>
-      <c r="B73" s="25">
+      <c r="B73" s="20">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"General (techniques / evaluation)",Included_102!$R$2:$R$103,"Lightweight")</f>
         <v/>
       </c>
-      <c r="C73" s="26">
+      <c r="C73" s="21">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"General (techniques / evaluation)",Included_102!$R$2:$R$103,"Compact")</f>
         <v/>
       </c>
-      <c r="D73" s="27">
+      <c r="D73" s="22">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"General (techniques / evaluation)",Included_102!$R$2:$R$103,"Moderate")</f>
         <v/>
       </c>
-      <c r="E73" s="28">
+      <c r="E73" s="23">
         <f>COUNTIFS(Included_102!$U$2:$U$103,"General (techniques / evaluation)",Included_102!$R$2:$R$103,"Higher")</f>
         <v/>
       </c>
@@ -15240,42 +14999,42 @@
         <f>COUNTIFS(Included_102!$U$2:$U$103,"General (techniques / evaluation)",Included_102!$R$2:$R$103,"Not stated")</f>
         <v/>
       </c>
-      <c r="H73" s="30">
+      <c r="H73" s="26">
         <f>SUM(B73:G73)</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="17" t="inlineStr">
+      <c r="A74" s="24" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B74" s="30">
+      <c r="B74" s="26">
         <f>SUM(B64:B73)</f>
         <v/>
       </c>
-      <c r="C74" s="30">
+      <c r="C74" s="26">
         <f>SUM(C64:C73)</f>
         <v/>
       </c>
-      <c r="D74" s="30">
+      <c r="D74" s="26">
         <f>SUM(D64:D73)</f>
         <v/>
       </c>
-      <c r="E74" s="30">
+      <c r="E74" s="26">
         <f>SUM(E64:E73)</f>
         <v/>
       </c>
-      <c r="F74" s="30">
+      <c r="F74" s="26">
         <f>SUM(F64:F73)</f>
         <v/>
       </c>
-      <c r="G74" s="30">
+      <c r="G74" s="26">
         <f>SUM(G64:G73)</f>
         <v/>
       </c>
-      <c r="H74" s="30">
+      <c r="H74" s="26">
         <f>SUM(H64:H73)</f>
         <v/>
       </c>
@@ -15314,7 +15073,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"United States")</f>
         <v/>
       </c>
-      <c r="C80" s="22">
+      <c r="C80" s="17">
         <f>B80/B$107</f>
         <v/>
       </c>
@@ -15329,7 +15088,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"China")</f>
         <v/>
       </c>
-      <c r="C81" s="22">
+      <c r="C81" s="17">
         <f>B81/B$107</f>
         <v/>
       </c>
@@ -15344,7 +15103,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"India")</f>
         <v/>
       </c>
-      <c r="C82" s="22">
+      <c r="C82" s="17">
         <f>B82/B$107</f>
         <v/>
       </c>
@@ -15359,7 +15118,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Germany")</f>
         <v/>
       </c>
-      <c r="C83" s="22">
+      <c r="C83" s="17">
         <f>B83/B$107</f>
         <v/>
       </c>
@@ -15374,7 +15133,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"South Korea")</f>
         <v/>
       </c>
-      <c r="C84" s="22">
+      <c r="C84" s="17">
         <f>B84/B$107</f>
         <v/>
       </c>
@@ -15389,7 +15148,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Saudi Arabia")</f>
         <v/>
       </c>
-      <c r="C85" s="22">
+      <c r="C85" s="17">
         <f>B85/B$107</f>
         <v/>
       </c>
@@ -15404,7 +15163,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Taiwan")</f>
         <v/>
       </c>
-      <c r="C86" s="22">
+      <c r="C86" s="17">
         <f>B86/B$107</f>
         <v/>
       </c>
@@ -15419,7 +15178,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Finland")</f>
         <v/>
       </c>
-      <c r="C87" s="22">
+      <c r="C87" s="17">
         <f>B87/B$107</f>
         <v/>
       </c>
@@ -15434,7 +15193,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"France")</f>
         <v/>
       </c>
-      <c r="C88" s="22">
+      <c r="C88" s="17">
         <f>B88/B$107</f>
         <v/>
       </c>
@@ -15449,7 +15208,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Singapore")</f>
         <v/>
       </c>
-      <c r="C89" s="22">
+      <c r="C89" s="17">
         <f>B89/B$107</f>
         <v/>
       </c>
@@ -15464,7 +15223,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Australia")</f>
         <v/>
       </c>
-      <c r="C90" s="22">
+      <c r="C90" s="17">
         <f>B90/B$107</f>
         <v/>
       </c>
@@ -15479,7 +15238,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Brazil")</f>
         <v/>
       </c>
-      <c r="C91" s="22">
+      <c r="C91" s="17">
         <f>B91/B$107</f>
         <v/>
       </c>
@@ -15494,7 +15253,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Bulgaria")</f>
         <v/>
       </c>
-      <c r="C92" s="22">
+      <c r="C92" s="17">
         <f>B92/B$107</f>
         <v/>
       </c>
@@ -15509,7 +15268,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Chile")</f>
         <v/>
       </c>
-      <c r="C93" s="22">
+      <c r="C93" s="17">
         <f>B93/B$107</f>
         <v/>
       </c>
@@ -15524,7 +15283,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Hungary")</f>
         <v/>
       </c>
-      <c r="C94" s="22">
+      <c r="C94" s="17">
         <f>B94/B$107</f>
         <v/>
       </c>
@@ -15539,7 +15298,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Israel")</f>
         <v/>
       </c>
-      <c r="C95" s="22">
+      <c r="C95" s="17">
         <f>B95/B$107</f>
         <v/>
       </c>
@@ -15554,7 +15313,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Italy")</f>
         <v/>
       </c>
-      <c r="C96" s="22">
+      <c r="C96" s="17">
         <f>B96/B$107</f>
         <v/>
       </c>
@@ -15569,7 +15328,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Netherlands")</f>
         <v/>
       </c>
-      <c r="C97" s="22">
+      <c r="C97" s="17">
         <f>B97/B$107</f>
         <v/>
       </c>
@@ -15584,7 +15343,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Nigeria")</f>
         <v/>
       </c>
-      <c r="C98" s="22">
+      <c r="C98" s="17">
         <f>B98/B$107</f>
         <v/>
       </c>
@@ -15599,7 +15358,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Norway")</f>
         <v/>
       </c>
-      <c r="C99" s="22">
+      <c r="C99" s="17">
         <f>B99/B$107</f>
         <v/>
       </c>
@@ -15614,7 +15373,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Pakistan")</f>
         <v/>
       </c>
-      <c r="C100" s="22">
+      <c r="C100" s="17">
         <f>B100/B$107</f>
         <v/>
       </c>
@@ -15629,7 +15388,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Qatar")</f>
         <v/>
       </c>
-      <c r="C101" s="22">
+      <c r="C101" s="17">
         <f>B101/B$107</f>
         <v/>
       </c>
@@ -15644,7 +15403,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"South Africa")</f>
         <v/>
       </c>
-      <c r="C102" s="22">
+      <c r="C102" s="17">
         <f>B102/B$107</f>
         <v/>
       </c>
@@ -15659,7 +15418,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Spain")</f>
         <v/>
       </c>
-      <c r="C103" s="22">
+      <c r="C103" s="17">
         <f>B103/B$107</f>
         <v/>
       </c>
@@ -15674,7 +15433,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Turkey")</f>
         <v/>
       </c>
-      <c r="C104" s="22">
+      <c r="C104" s="17">
         <f>B104/B$107</f>
         <v/>
       </c>
@@ -15689,7 +15448,7 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"United Kingdom")</f>
         <v/>
       </c>
-      <c r="C105" s="22">
+      <c r="C105" s="17">
         <f>B105/B$107</f>
         <v/>
       </c>
@@ -15704,33 +15463,33 @@
         <f>COUNTIF(Included_102!$Z$2:$Z$103,"Vietnam")</f>
         <v/>
       </c>
-      <c r="C106" s="22">
+      <c r="C106" s="17">
         <f>B106/B$107</f>
         <v/>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="23" t="inlineStr">
+      <c r="A107" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B107" s="23">
+      <c r="B107" s="18">
         <f>SUM(B80:B106)</f>
         <v/>
       </c>
-      <c r="C107" s="24">
+      <c r="C107" s="19">
         <f>B107/B107</f>
         <v/>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="17" t="inlineStr">
+      <c r="A108" s="24" t="inlineStr">
         <is>
           <t>Countries represented</t>
         </is>
       </c>
-      <c r="B108" s="29">
+      <c r="B108" s="25">
         <f>SUMPRODUCT(1/COUNTIF(Included_102!$Z$2:$Z$103,Included_102!$Z$2:$Z$103))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add link for Wang (2025)
</commit_message>
<xml_diff>
--- a/SLM_Review_Dataset.xlsx
+++ b/SLM_Review_Dataset.xlsx
@@ -11726,7 +11726,11 @@
           <t>Preprint (author website)</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr"/>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>https://pics.iamzhaokun.com/doc/report/Resource-Efficient%20Knowledge%20Distillation%20for%20Qwen2.5-0.5B-Instruct.pdf</t>
+        </is>
+      </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
           <t>Preprint</t>
@@ -12676,13 +12680,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G103" r:id="rId102"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix title formatting and header colour
</commit_message>
<xml_diff>
--- a/SLM_Review_Dataset.xlsx
+++ b/SLM_Review_Dataset.xlsx
@@ -36,7 +36,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001B2329"/>
       <sz val="11"/>
     </font>
     <font>
@@ -63,7 +63,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="001B2329"/>
     </font>
     <font>
       <i val="1"/>
@@ -71,7 +71,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -80,7 +80,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A5F"/>
+        <fgColor rgb="00EEF1F3"/>
       </patternFill>
     </fill>
     <fill>
@@ -106,11 +106,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDF4FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EEF1F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -177,15 +172,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1235,7 +1230,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Optimizing RAG techniques for automotive industry PDF chatbots: A case study with locally deployed Ollama models</t>
+          <t>Optimizing RAG Techniques for Automotive Industry PDF Chatbots: A Case Study with Locally Deployed Ollama Models</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -1343,7 +1338,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Improving small language models on pubmedqa via generative data augmentation</t>
+          <t>Improving Small Language Models on PubMedQA via Generative Data Augmentation</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -1459,7 +1454,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>MedMobile: A mobile-sized language model with clinical capabilities</t>
+          <t>MedMobile: A Mobile-Sized Language Model with Clinical Capabilities</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -1687,7 +1682,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Modeling legal reasoning: Lm annotation at the edge of human agreement</t>
+          <t>Modeling Legal Reasoning: LM Annotation at the Edge of Human Agreement</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -1799,7 +1794,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Synthesizing question answering data from financial documents: An End-to-End Multi-Agent Approach</t>
+          <t>Synthesizing Question Answering Data from Financial Documents: An End-to-End Multi-Agent Approach</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -2023,7 +2018,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Flame: A small language model for spreadsheet formulas</t>
+          <t>FLAME: A Small Language Model for Spreadsheet Formulas</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
@@ -2135,7 +2130,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Chain-of-thought in neural code generation: From and for lightweight language models</t>
+          <t>Chain-of-Thought in Neural Code Generation: From and For Lightweight Language Models</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -2247,7 +2242,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Perfrl: A small language model framework for efficient code optimization</t>
+          <t>PerfRL: A Small Language Model Framework for Efficient Code Optimization</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -2475,7 +2470,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Assessing small language models for code generation: An empirical study with benchmarks</t>
+          <t>Assessing Small Language Models for Code Generation: An Empirical Study with Benchmarks</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -2587,7 +2582,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Datagpt-sql-7b: An open-source language model for text-to-sql</t>
+          <t>DataGpt-SQL-7B: An Open-Source Language Model for Text-to-SQL</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -2823,7 +2818,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>TinyRS-R1: Compact vision language model for remote sensing</t>
+          <t>TinyRS-R1: Compact Vision Language Model for Remote Sensing</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -2935,7 +2930,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Exploring lightweight language models for materials informatics with AlchemBERT</t>
+          <t>Exploring Lightweight Language Models for Materials Informatics with AlchemBERT</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -3047,7 +3042,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>PepBERT: Lightweight language models for bioactive peptide representation</t>
+          <t>PepBERT: Lightweight Language Models for Bioactive Peptide Representation</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
@@ -3159,7 +3154,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>AdaVITS: Tiny VITS for low computing resource speaker adaptation</t>
+          <t>AdaVITS: Tiny VITS for Low Computing Resource Speaker Adaptation</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -3271,7 +3266,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>A compact end-to-end model with local and global context for spoken language identification</t>
+          <t>A Compact End-to-End Model with Local and Global Context for Spoken Language Identification</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
@@ -3735,7 +3730,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Mellow: a small audio language model for reasoning</t>
+          <t>Mellow: A Small Audio Language Model for Reasoning</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -3847,7 +3842,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Distilling on-device language models for robot planning with minimal human intervention</t>
+          <t>Distilling On-Device Language Models for Robot Planning with Minimal Human Intervention</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -3963,7 +3958,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Transformer-lite: High-efficiency deployment of large language models on mobile phone gpus</t>
+          <t>Transformer-Lite: High-Efficiency Deployment of Large Language Models on Mobile Phone GPUs</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
@@ -4079,7 +4074,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Edge-first language model inference: Models, metrics, and tradeoffs</t>
+          <t>Edge-First Language Model Inference: Models, Metrics, and Tradeoffs</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
@@ -4303,7 +4298,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>$\$CLONE$\$: Customizing $\$LLMs$\$ for Efficient $\$Latency-Aware$\$ Inference at the Edge</t>
+          <t>CLONE: Customizing LLMs for Efficient Latency-Aware Inference at the Edge</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
@@ -4415,7 +4410,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Swahbert: Language model of swahili</t>
+          <t>SwahBERT: Language Model of Swahili</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
@@ -4527,7 +4522,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Inkubalm: A small language model for low-resource african languages</t>
+          <t>InkubaLM: A Small Language Model for Low-Resource African Languages</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
@@ -4991,7 +4986,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>BERTabaporu: assessing a genre-specific language model for Portuguese NLP</t>
+          <t>BERTabaporu: Assessing a Genre-Specific Language Model for Portuguese NLP</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
@@ -5103,7 +5098,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>mALBERT: Is a compact multilingual bert model still worth it?</t>
+          <t>mALBERT: Is a Compact Multilingual BERT Model Still Worth It?</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
@@ -5787,7 +5782,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>UniGen: Universal domain generalization for sentiment classification via zero-shot dataset generation</t>
+          <t>UniGen: Universal Domain Generalization for Sentiment Classification via Zero-Shot Dataset Generation</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
@@ -5899,7 +5894,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Tiny language models enriched with multimodal knowledge from multiplex networks</t>
+          <t>Tiny Language Models Enriched with Multimodal Knowledge from Multiplex Networks</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
@@ -6127,7 +6122,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Octopus v2: On-device language model for super agent</t>
+          <t>Octopus v2: On-Device Language Model for Super Agent</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
@@ -7859,7 +7854,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Could small language models serve as recommenders? towards data-centric cold-start recommendation</t>
+          <t>Could Small Language Models Serve as Recommenders? Towards Data-centric Cold-start Recommendations</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
@@ -8083,7 +8078,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Shakti: A 2.5 billion parameter small language model optimized for edge ai and low-resource environments</t>
+          <t>SHAKTI: A 2.5 Billion Parameter Small Language Model Optimized for Edge AI and Low-Resource Environments</t>
         </is>
       </c>
       <c r="E63" s="2" t="n">
@@ -8535,7 +8530,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Adaptive multitask emotion recognition and sentiment analysis using resource-constrained MobileBERT and DistilBERT: an efficient approach for edge devices</t>
+          <t>Adaptive Multitask Emotion Recognition and Sentiment Analysis Using Resource-Constrained MobileBERT and DistilBERT: An Efficient Approach for Edge Devices</t>
         </is>
       </c>
       <c r="E67" s="2" t="n">
@@ -8755,7 +8750,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Mobilellm: Optimizing sub-billion parameter language models for on-device use cases</t>
+          <t>MobileLLM: Optimizing Sub-billion Parameter Language Models for On-Device Use Cases</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
@@ -8971,7 +8966,7 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>On-device Qwen2. 5: Efficient LLM inference with model compression and hardware acceleration</t>
+          <t>On-Device Qwen2.5: Efficient LLM Inference with Model Compression and Hardware Acceleration</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
@@ -9411,7 +9406,7 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>How does GPT-2 compute greater-than?: Interpreting mathematical abilities in a pre-trained language model</t>
+          <t>How Does GPT-2 Compute Greater-Than?: Interpreting Mathematical Abilities in a Pre-Trained Language Model</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
@@ -9951,7 +9946,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Nextcoder: Robust adaptation of code LMs to diverse code edits</t>
+          <t>NextCoder: Robust Adaptation of Code LMs to Diverse Code Edits</t>
         </is>
       </c>
       <c r="E80" s="2" t="n">
@@ -10395,7 +10390,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Locally-deployed vs. cloud-based AI in healthcare: evaluating DeepSeek-R1: 8b, DeepSeek-R1, and ChatGPT o3-mini-high for complex medical diagnostics</t>
+          <t>Locally-Deployed vs. Cloud-Based AI in Healthcare: Evaluating DeepSeek-R1:8b, DeepSeek-R1, and ChatGPT o3-mini-high for Complex Medical Diagnostics</t>
         </is>
       </c>
       <c r="E84" s="2" t="n">
@@ -10731,7 +10726,7 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Compact language models via pruning and knowledge distillation</t>
+          <t>Compact Language Models via Pruning and Knowledge Distillation</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
@@ -10839,7 +10834,7 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Quantized transformer language model implementations on edge devices</t>
+          <t>Quantized Transformer Language Model Implementations on Edge Devices</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
@@ -11055,7 +11050,7 @@
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Judgeboard: Benchmarking and enhancing small language models for reasoning evaluation</t>
+          <t>JudgeBoard: Benchmarking and Enhancing Small Language Models for Reasoning Evaluation</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
@@ -11495,7 +11490,7 @@
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Orca 2: Teaching small language models how to reason</t>
+          <t>Orca 2: Teaching Small Language Models How to Reason</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
@@ -11607,7 +11602,7 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Distilqwen2. 5: Industrial practices of training distilled open lightweight language models</t>
+          <t>DistilQwen2.5: Industrial Practices of Training Distilled Open Lightweight Language Models</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
@@ -11831,7 +11826,7 @@
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Small models struggle to learn from strong reasoners</t>
+          <t>Small Models Struggle to Learn from Strong Reasoners</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
@@ -12163,7 +12158,7 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>An emulator for fine-tuning large language models using small language models</t>
+          <t>An Emulator for Fine-Tuning Large Language Models using Small Language Models</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
@@ -12383,7 +12378,7 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Can small language models help large language models reason better?: LM-guided chain-of-thought</t>
+          <t>Can Small Language Models Help Large Language Models Reason Better?: LM-Guided Chain-of-Thought</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
@@ -12491,7 +12486,7 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Adaptivelog: An adaptive log analysis framework with the collaboration of large and small language model</t>
+          <t>AdaptiveLog: An Adaptive Log Analysis Framework with the Collaboration of Large and Small Language Model</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
@@ -13091,7 +13086,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Analyzing distilbert for sentiment classification of banking financial news</t>
+          <t>Analyzing DistilBERT for Sentiment Classification of Banking Financial News</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -13226,7 +13221,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>ChatGPT vs. DeepSeek: A comparative study on AI-based code generation</t>
+          <t>ChatGPT vs. DeepSeek: A Comparative Study on AI-Based Code Generation</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -13361,7 +13356,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>A method for the architecture of a medical vertical large language model based on deepseek r1</t>
+          <t>A Method for the Architecture of a Medical Vertical Large Language Model Based on DeepSeek R1</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -13406,7 +13401,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Token-hungry, yet precise: Deepseek r1 highlights the need for multi-step reasoning over speed in math</t>
+          <t>Token-Hungry, Yet Precise: DeepSeek R1 Highlights the Need for Multi-Step Reasoning Over Speed in MATH</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -13496,7 +13491,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Fine-tuning mistral 7b large language model for python query response and code generation: A parameter efficient approach</t>
+          <t>Fine-Tuning Mistral 7B Large Language Model for Python Query Response and Code Generation: A Parameter Efficient Approach</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update reference numbers to the revised article; SlimLM now cited in its ACL 2025 version
</commit_message>
<xml_diff>
--- a/SLM_Review_Dataset.xlsx
+++ b/SLM_Review_Dataset.xlsx
@@ -418,7 +418,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Application domain (Figure 4; Table 4 = domain-specific)</a:t>
+              <a:t>Application domain (Figure 4, Tables 4–5)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3140,7 +3140,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -3368,7 +3368,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -3484,7 +3484,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
@@ -3600,7 +3600,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -3716,7 +3716,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -3828,7 +3828,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -3944,7 +3944,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -4060,7 +4060,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -4172,7 +4172,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -4284,7 +4284,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -4396,7 +4396,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -4508,7 +4508,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -4628,7 +4628,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -4744,7 +4744,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -4856,7 +4856,7 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -4972,7 +4972,7 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
@@ -5084,7 +5084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -5196,7 +5196,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
@@ -5316,7 +5316,7 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -5432,7 +5432,7 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
@@ -5544,7 +5544,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -5656,7 +5656,7 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -5880,7 +5880,7 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
@@ -5992,7 +5992,7 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -6108,7 +6108,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
@@ -6228,7 +6228,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
@@ -6344,7 +6344,7 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
@@ -6460,7 +6460,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
@@ -6576,7 +6576,7 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
@@ -6688,7 +6688,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
@@ -6804,7 +6804,7 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
@@ -6920,7 +6920,7 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
@@ -7036,7 +7036,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
@@ -7264,11 +7264,11 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>pham2024slimlm</t>
+          <t>pham2025slimlm</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -7291,27 +7291,27 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2411.09944</t>
+          <t>https://doi.org/10.18653/v1/2025.acl-demo.42</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Preprint</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr"/>
+          <t>Peer-reviewed</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Published version: ACL 2025 (System Demonstrations)</t>
+        </is>
+      </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>b (16)</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M56" s="2" t="inlineStr"/>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
+      <c r="M56" s="2" t="n"/>
       <c r="N56" s="3" t="inlineStr">
         <is>
           <t>SlimLM</t>
@@ -7380,7 +7380,7 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
@@ -7492,7 +7492,7 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
@@ -7608,7 +7608,7 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
@@ -7724,7 +7724,7 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
@@ -7840,7 +7840,7 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
@@ -7952,7 +7952,7 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
@@ -8064,7 +8064,7 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
@@ -8176,7 +8176,7 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
@@ -8292,7 +8292,7 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
@@ -8404,7 +8404,7 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
@@ -8516,7 +8516,7 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
@@ -8624,7 +8624,7 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
@@ -8736,7 +8736,7 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
@@ -8844,7 +8844,7 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
@@ -8952,7 +8952,7 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
@@ -9064,7 +9064,7 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
@@ -9500,7 +9500,7 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
@@ -9608,7 +9608,7 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
@@ -9716,7 +9716,7 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
@@ -9824,7 +9824,7 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
@@ -9932,7 +9932,7 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>130</v>
+        <v>105</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
@@ -10040,7 +10040,7 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
@@ -10156,7 +10156,7 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>136</v>
+        <v>101</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
@@ -10268,7 +10268,7 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
@@ -10376,7 +10376,7 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
@@ -10484,7 +10484,7 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
@@ -10596,7 +10596,7 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>150</v>
+        <v>122</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
@@ -10712,7 +10712,7 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
@@ -10820,7 +10820,7 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
@@ -10928,7 +10928,7 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>159</v>
+        <v>124</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
@@ -11036,7 +11036,7 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>160</v>
+        <v>125</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
@@ -11144,7 +11144,7 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>162</v>
+        <v>126</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
@@ -11252,7 +11252,7 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>163</v>
+        <v>127</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
@@ -11364,7 +11364,7 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>164</v>
+        <v>128</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
@@ -11476,7 +11476,7 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>177</v>
+        <v>129</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
@@ -11588,7 +11588,7 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>178</v>
+        <v>130</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
@@ -11696,7 +11696,7 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>179</v>
+        <v>131</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
@@ -11812,7 +11812,7 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>180</v>
+        <v>132</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
@@ -11920,7 +11920,7 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>183</v>
+        <v>133</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
@@ -12028,7 +12028,7 @@
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>186</v>
+        <v>134</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
@@ -12144,7 +12144,7 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>189</v>
+        <v>135</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
@@ -12256,7 +12256,7 @@
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>190</v>
+        <v>136</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
@@ -12364,7 +12364,7 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>191</v>
+        <v>137</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
@@ -12472,7 +12472,7 @@
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>192</v>
+        <v>106</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
@@ -12847,7 +12847,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -12892,7 +12892,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -12937,7 +12937,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -12982,7 +12982,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -13027,7 +13027,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -13072,7 +13072,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>103</v>
+        <v>141</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -13117,7 +13117,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -13162,7 +13162,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -13207,7 +13207,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -13252,7 +13252,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -13297,7 +13297,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -13342,7 +13342,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -13387,7 +13387,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -13432,7 +13432,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -13477,7 +13477,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -13522,7 +13522,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -14246,7 +14246,7 @@
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>Application domain (Figure 4; Table 4 = domain-specific)</t>
+          <t>Application domain (Figure 4, Tables 4–5)</t>
         </is>
       </c>
     </row>
@@ -14435,7 +14435,7 @@
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>Domain-specific (Table 4)</t>
+          <t>Domain-specific (Figure 4)</t>
         </is>
       </c>
       <c r="B38" s="25">

</xml_diff>